<commit_message>
n8n board refresh 2026-10-29T17:41:49Z
</commit_message>
<xml_diff>
--- a/app/reports/BPRE_research.xlsx
+++ b/app/reports/BPRE_research.xlsx
@@ -615,7 +615,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-10-28 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
+          <t>Generated 2026-10-29 17:35 · Source: FMP · Methodology: financial-analysis plugin (Anthropic FSI), adapted for free-tier data</t>
         </is>
       </c>
     </row>
@@ -686,7 +686,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>12.465</v>
+        <v>12.385</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>0.05015999794006348</v>
+        <v>0.04994999885559082</v>
       </c>
     </row>
     <row r="6">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="B35" s="18" t="n">
-        <v>143044369.3541918</v>
+        <v>143044366.5724667</v>
       </c>
     </row>
     <row r="36">
@@ -1200,7 +1200,7 @@
         </is>
       </c>
       <c r="B37" s="20" t="n">
-        <v>12.465</v>
+        <v>12.385</v>
       </c>
     </row>
     <row r="38">
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="C5" s="28" t="n">
-        <v>1783048064</v>
+        <v>1771604480</v>
       </c>
       <c r="D5" s="29" t="n"/>
       <c r="E5" s="29" t="n"/>

</xml_diff>